<commit_message>
Solver, import data from pdf,goal seek, scenario
</commit_message>
<xml_diff>
--- a/11. Dynamic Dropdown LIst/dynamic_list.xlsx
+++ b/11. Dynamic Dropdown LIst/dynamic_list.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Advance_Excel_BI\11. Dynamic Dropdown LIst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23177498-8DF0-4221-847F-6ADDCE348501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3E54FE-780B-41B8-8EA9-91C1E3C8B4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{DFBDDC44-5B26-4933-9FE5-39F5FC447B3C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{DFBDDC44-5B26-4933-9FE5-39F5FC447B3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic_List_or_Dependent _Drop" sheetId="4" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Australia">'Dynamic_List_or_Dependent _Drop'!$K$9</definedName>
-    <definedName name="Canada">'Dynamic_List_or_Dependent _Drop'!$J$9:$J$11</definedName>
-    <definedName name="China">'Dynamic_List_or_Dependent _Drop'!$I$9:$I$11</definedName>
-    <definedName name="India">'Dynamic_List_or_Dependent _Drop'!$G$9:$G$13</definedName>
-    <definedName name="Malaysia">'Dynamic_List_or_Dependent _Drop'!$H$9:$H$11</definedName>
+    <definedName name="Australia">Sheet1!$H$5</definedName>
+    <definedName name="Canada">Sheet1!$G$5:$G$7</definedName>
+    <definedName name="China">Sheet1!$F$5:$F$7</definedName>
+    <definedName name="India">Sheet1!$D$5:$D$10</definedName>
+    <definedName name="Malaysia">Sheet1!$E$5:$E$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="29">
   <si>
     <t>India</t>
   </si>
@@ -127,6 +128,21 @@
   </si>
   <si>
     <t>Sydney</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Institute Country Location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Institute city </t>
+  </si>
+  <si>
+    <t>IBM</t>
+  </si>
+  <si>
+    <t>Ahmedabad</t>
   </si>
 </sst>
 </file>
@@ -170,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -178,6 +194,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -668,10 +687,10 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="N16" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O16" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -698,4 +717,131 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65D51D75-D860-4032-9BA0-A95243AA4163}">
+  <dimension ref="C3:P11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="22.5546875" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="3:16" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="3:16" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="O9" t="s">
+        <v>0</v>
+      </c>
+      <c r="P9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="O10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="3:16" x14ac:dyDescent="0.3">
+      <c r="J11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11">
+        <v>178</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O9:O21" xr:uid="{5518C114-5328-4D61-9D24-B28F73304AEC}">
+      <formula1>$D$4:$H$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P9:P21" xr:uid="{E5B68250-CC84-4E90-8293-35176744D5AE}">
+      <formula1>INDIRECT($O$9)</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>